<commit_message>
ci: update Phase 7 GitHub Actions deployment and E2E test suite
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Passed_Test_Cases.xlsx
+++ b/automation/reports/Excel/Passed_Test_Cases.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7.001</v>
+        <v>25.774</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.224</v>
+        <v>0.236</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.189</v>
+        <v>0.288</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.239</v>
+        <v>0.218</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.182</v>
+        <v>0.31</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.369</v>
+        <v>0.242</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.275</v>
+        <v>0.332</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.317</v>
+        <v>0.258</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.374</v>
+        <v>0.445</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.315</v>
+        <v>0.506</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.181</v>
+        <v>0.308</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.217</v>
+        <v>0.29</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.203</v>
+        <v>0.295</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.21</v>
+        <v>0.279</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.168</v>
+        <v>0.228</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.225</v>
+        <v>0.265</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.178</v>
+        <v>0.249</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.227</v>
+        <v>0.248</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.167</v>
+        <v>0.262</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.22</v>
+        <v>0.239</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.172</v>
+        <v>0.218</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.213</v>
+        <v>0.26</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.169</v>
+        <v>0.229</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.207</v>
+        <v>0.216</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.166</v>
+        <v>0.27</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.212</v>
+        <v>0.24</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.175</v>
+        <v>0.224</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.225</v>
+        <v>0.265</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.18</v>
+        <v>0.243</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.207</v>
+        <v>0.224</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.177</v>
+        <v>0.276</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.213</v>
+        <v>0.243</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.18</v>
+        <v>0.239</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.221</v>
+        <v>0.266</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.172</v>
+        <v>0.245</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.217</v>
+        <v>0.248</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.174</v>
+        <v>0.328</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.215</v>
+        <v>0.293</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.168</v>
+        <v>0.239</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.214</v>
+        <v>0.253</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>3.46</v>
+        <v>14.577</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.258</v>
+        <v>0.325</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.378</v>
+        <v>0.577</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.222</v>
+        <v>0.349</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.276</v>
+        <v>0.337</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.224</v>
+        <v>0.269</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.253</v>
+        <v>0.258</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.211</v>
+        <v>0.231</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.255</v>
+        <v>0.278</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.209</v>
+        <v>0.266</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.246</v>
+        <v>0.307</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.222</v>
+        <v>0.292</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.253</v>
+        <v>0.297</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.225</v>
+        <v>0.303</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.25</v>
+        <v>0.273</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.216</v>
+        <v>0.27</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.255</v>
+        <v>0.218</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.216</v>
+        <v>0.265</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.252</v>
+        <v>0.259</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.226</v>
+        <v>0.312</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.289</v>
+        <v>0.268</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -2338,7 +2338,7 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.292</v>
+        <v>0.25</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.227</v>
+        <v>0.287</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.21</v>
+        <v>0.276</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0.251</v>
+        <v>0.254</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.216</v>
+        <v>0.291</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -2488,7 +2488,7 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.266</v>
+        <v>0.271</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.211</v>
+        <v>0.266</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.257</v>
+        <v>0.303</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -2578,7 +2578,7 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0.229</v>
+        <v>0.277</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -2608,7 +2608,7 @@
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.25</v>
+        <v>0.218</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0.215</v>
+        <v>0.294</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -2668,7 +2668,7 @@
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.248</v>
+        <v>0.282</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>0.22</v>
+        <v>0.252</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>0.258</v>
+        <v>0.297</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.214</v>
+        <v>0.285</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -2788,7 +2788,7 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.254</v>
+        <v>0.248</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -2818,7 +2818,7 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0.212</v>
+        <v>0.261</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.256</v>
+        <v>0.276</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0.211</v>
+        <v>0.263</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -2908,7 +2908,7 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>3.378</v>
+        <v>5.068</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.36</v>
+        <v>0.437</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -2968,7 +2968,7 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>0.373</v>
+        <v>0.421</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>0.34</v>
+        <v>0.442</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>0.288</v>
+        <v>0.274</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -3058,7 +3058,7 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0.23</v>
+        <v>0.255</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -3088,7 +3088,7 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>0.251</v>
+        <v>0.37</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -3118,7 +3118,7 @@
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>0.21</v>
+        <v>0.257</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>0.257</v>
+        <v>0.43</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -3178,7 +3178,7 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0.214</v>
+        <v>0.331</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>0.265</v>
+        <v>0.323</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -3238,7 +3238,7 @@
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>0.206</v>
+        <v>0.31</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -3268,7 +3268,7 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0.253</v>
+        <v>0.316</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0.219</v>
+        <v>0.302</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>0.249</v>
+        <v>0.296</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>0.21</v>
+        <v>0.294</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -3388,7 +3388,7 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0.25</v>
+        <v>0.29</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>0.215</v>
+        <v>0.303</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>0.242</v>
+        <v>0.292</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -3478,7 +3478,7 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0.209</v>
+        <v>0.301</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>0.242</v>
+        <v>0.311</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -3538,7 +3538,7 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>0.21</v>
+        <v>0.304</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -3568,7 +3568,7 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>0.247</v>
+        <v>0.328</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>0.216</v>
+        <v>0.293</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0.249</v>
+        <v>0.268</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>0.208</v>
+        <v>0.303</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -3688,7 +3688,7 @@
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>0.198</v>
+        <v>0.274</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>0.275</v>
+        <v>0.292</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>0.226</v>
+        <v>0.534</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -3778,7 +3778,7 @@
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>0.261</v>
+        <v>0.305</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="E112" s="2" t="n">
-        <v>5.556</v>
+        <v>4.609</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -3838,7 +3838,7 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0.294</v>
+        <v>0.382</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>0.251</v>
+        <v>0.648</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0.242</v>
+        <v>0.466</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -3928,7 +3928,7 @@
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0.112</v>
+        <v>0.331</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>0.262</v>
+        <v>0.242</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>0.271</v>
+        <v>0.232</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -4018,7 +4018,7 @@
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0.216</v>
+        <v>0.34</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0.252</v>
+        <v>0.336</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -4078,7 +4078,7 @@
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>0.219</v>
+        <v>0.32</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>0.26</v>
+        <v>0.375</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>0.216</v>
+        <v>0.401</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -4168,7 +4168,7 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>0.248</v>
+        <v>0.284</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="E125" s="2" t="n">
-        <v>0.218</v>
+        <v>0.43</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -4228,7 +4228,7 @@
         </is>
       </c>
       <c r="E126" s="2" t="n">
-        <v>0.216</v>
+        <v>0.362</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -4258,7 +4258,7 @@
         </is>
       </c>
       <c r="E127" s="2" t="n">
-        <v>0.26</v>
+        <v>0.232</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -4288,7 +4288,7 @@
         </is>
       </c>
       <c r="E128" s="2" t="n">
-        <v>0.214</v>
+        <v>0.334</v>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
@@ -4318,7 +4318,7 @@
         </is>
       </c>
       <c r="E129" s="2" t="n">
-        <v>0.243</v>
+        <v>0.328</v>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="E130" s="2" t="n">
-        <v>0.213</v>
+        <v>0.315</v>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
@@ -4378,7 +4378,7 @@
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>0.255</v>
+        <v>0.382</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>0.212</v>
+        <v>0.322</v>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>0.254</v>
+        <v>0.285</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -4468,7 +4468,7 @@
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>0.223</v>
+        <v>0.256</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>0.255</v>
+        <v>0.295</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -4528,7 +4528,7 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>0.222</v>
+        <v>0.279</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -4558,7 +4558,7 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>0.29</v>
+        <v>0.256</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>0.211</v>
+        <v>0.298</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -4618,7 +4618,7 @@
         </is>
       </c>
       <c r="E139" s="2" t="n">
-        <v>0.262</v>
+        <v>0.275</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>0.208</v>
+        <v>0.258</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -4678,7 +4678,7 @@
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>0.263</v>
+        <v>0.314</v>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>0.216</v>
+        <v>0.296</v>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
@@ -4738,7 +4738,7 @@
         </is>
       </c>
       <c r="E143" s="2" t="n">
-        <v>0.281</v>
+        <v>0.274</v>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="E144" s="2" t="n">
-        <v>0.219</v>
+        <v>0.304</v>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
         </is>
       </c>
       <c r="E145" s="2" t="n">
-        <v>0.321</v>
+        <v>0.277</v>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
@@ -4828,7 +4828,7 @@
         </is>
       </c>
       <c r="E146" s="2" t="n">
-        <v>0.248</v>
+        <v>0.252</v>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="E147" s="2" t="n">
-        <v>0.222</v>
+        <v>0.299</v>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
@@ -4888,7 +4888,7 @@
         </is>
       </c>
       <c r="E148" s="2" t="n">
-        <v>0.224</v>
+        <v>0.272</v>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
@@ -4918,7 +4918,7 @@
         </is>
       </c>
       <c r="E149" s="2" t="n">
-        <v>0.252</v>
+        <v>0.26</v>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
         </is>
       </c>
       <c r="E150" s="2" t="n">
-        <v>0.22</v>
+        <v>0.303</v>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
@@ -4978,7 +4978,7 @@
         </is>
       </c>
       <c r="E151" s="2" t="n">
-        <v>0.262</v>
+        <v>0.273</v>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="E152" s="2" t="n">
-        <v>0.24</v>
+        <v>0.257</v>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
         </is>
       </c>
       <c r="E153" s="2" t="n">
-        <v>0.261</v>
+        <v>0.308</v>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
@@ -5068,7 +5068,7 @@
         </is>
       </c>
       <c r="E154" s="2" t="n">
-        <v>0.212</v>
+        <v>0.28</v>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="E155" s="2" t="n">
-        <v>0.267</v>
+        <v>0.265</v>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
@@ -5128,7 +5128,7 @@
         </is>
       </c>
       <c r="E156" s="2" t="n">
-        <v>0.217</v>
+        <v>0.308</v>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
@@ -5158,7 +5158,7 @@
         </is>
       </c>
       <c r="E157" s="2" t="n">
-        <v>0.252</v>
+        <v>0.28</v>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
@@ -5188,7 +5188,7 @@
         </is>
       </c>
       <c r="E158" s="2" t="n">
-        <v>0.219</v>
+        <v>0.275</v>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
@@ -5218,7 +5218,7 @@
         </is>
       </c>
       <c r="E159" s="2" t="n">
-        <v>0.249</v>
+        <v>0.318</v>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
         </is>
       </c>
       <c r="E160" s="2" t="n">
-        <v>0.233</v>
+        <v>0.274</v>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
@@ -5278,7 +5278,7 @@
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>0.265</v>
+        <v>0.276</v>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         </is>
       </c>
       <c r="E162" s="2" t="n">
-        <v>10.929</v>
+        <v>4.643</v>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
@@ -5338,7 +5338,7 @@
         </is>
       </c>
       <c r="E163" s="2" t="n">
-        <v>0.298</v>
+        <v>0.336</v>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
@@ -5368,7 +5368,7 @@
         </is>
       </c>
       <c r="E164" s="2" t="n">
-        <v>0.325</v>
+        <v>0.312</v>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
         </is>
       </c>
       <c r="E165" s="2" t="n">
-        <v>0.219</v>
+        <v>0.301</v>
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
@@ -5428,7 +5428,7 @@
         </is>
       </c>
       <c r="E166" s="2" t="n">
-        <v>0.261</v>
+        <v>0.31</v>
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
@@ -5458,7 +5458,7 @@
         </is>
       </c>
       <c r="E167" s="2" t="n">
-        <v>0.217</v>
+        <v>0.282</v>
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
@@ -5488,7 +5488,7 @@
         </is>
       </c>
       <c r="E168" s="2" t="n">
-        <v>0.26</v>
+        <v>0.227</v>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
@@ -5518,7 +5518,7 @@
         </is>
       </c>
       <c r="E169" s="2" t="n">
-        <v>0.224</v>
+        <v>0.282</v>
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
         </is>
       </c>
       <c r="E170" s="2" t="n">
-        <v>0.266</v>
+        <v>0.326</v>
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
@@ -5578,7 +5578,7 @@
         </is>
       </c>
       <c r="E171" s="2" t="n">
-        <v>0.195</v>
+        <v>0.278</v>
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
@@ -5608,7 +5608,7 @@
         </is>
       </c>
       <c r="E172" s="2" t="n">
-        <v>0.258</v>
+        <v>0.306</v>
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
@@ -5638,7 +5638,7 @@
         </is>
       </c>
       <c r="E173" s="2" t="n">
-        <v>0.214</v>
+        <v>0.251</v>
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
@@ -5668,7 +5668,7 @@
         </is>
       </c>
       <c r="E174" s="2" t="n">
-        <v>0.267</v>
+        <v>0.304</v>
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
         </is>
       </c>
       <c r="E175" s="2" t="n">
-        <v>0.196</v>
+        <v>0.266</v>
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
@@ -5728,7 +5728,7 @@
         </is>
       </c>
       <c r="E176" s="2" t="n">
-        <v>0.245</v>
+        <v>0.318</v>
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
@@ -5758,7 +5758,7 @@
         </is>
       </c>
       <c r="E177" s="2" t="n">
-        <v>0.211</v>
+        <v>0.257</v>
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
@@ -5788,7 +5788,7 @@
         </is>
       </c>
       <c r="E178" s="2" t="n">
-        <v>0.267</v>
+        <v>0.307</v>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
@@ -5818,7 +5818,7 @@
         </is>
       </c>
       <c r="E179" s="2" t="n">
-        <v>0.224</v>
+        <v>0.254</v>
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
         </is>
       </c>
       <c r="E180" s="2" t="n">
-        <v>0.288</v>
+        <v>0.307</v>
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
@@ -5878,7 +5878,7 @@
         </is>
       </c>
       <c r="E181" s="2" t="n">
-        <v>0.222</v>
+        <v>0.252</v>
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         </is>
       </c>
       <c r="E182" s="2" t="n">
-        <v>0.284</v>
+        <v>0.305</v>
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
@@ -5938,7 +5938,7 @@
         </is>
       </c>
       <c r="E183" s="2" t="n">
-        <v>0.217</v>
+        <v>0.266</v>
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
@@ -5968,7 +5968,7 @@
         </is>
       </c>
       <c r="E184" s="2" t="n">
-        <v>0.26</v>
+        <v>0.304</v>
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
         </is>
       </c>
       <c r="E185" s="2" t="n">
-        <v>0.225</v>
+        <v>0.267</v>
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="E186" s="2" t="n">
-        <v>0.272</v>
+        <v>0.299</v>
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
@@ -6058,7 +6058,7 @@
         </is>
       </c>
       <c r="E187" s="2" t="n">
-        <v>0.223</v>
+        <v>0.25</v>
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
@@ -6088,7 +6088,7 @@
         </is>
       </c>
       <c r="E188" s="2" t="n">
-        <v>0.292</v>
+        <v>0.317</v>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
@@ -6118,7 +6118,7 @@
         </is>
       </c>
       <c r="E189" s="2" t="n">
-        <v>0.256</v>
+        <v>0.252</v>
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
         </is>
       </c>
       <c r="E190" s="2" t="n">
-        <v>0.244</v>
+        <v>0.304</v>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="E191" s="2" t="n">
-        <v>0.211</v>
+        <v>0.251</v>
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
@@ -6208,7 +6208,7 @@
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>0.269</v>
+        <v>0.352</v>
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
@@ -6238,7 +6238,7 @@
         </is>
       </c>
       <c r="E193" s="2" t="n">
-        <v>0.229</v>
+        <v>0.259</v>
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         </is>
       </c>
       <c r="E194" s="2" t="n">
-        <v>0.263</v>
+        <v>0.304</v>
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
         </is>
       </c>
       <c r="E195" s="2" t="n">
-        <v>0.22</v>
+        <v>0.248</v>
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="E196" s="2" t="n">
-        <v>0.268</v>
+        <v>0.299</v>
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="E197" s="2" t="n">
-        <v>0.216</v>
+        <v>0.248</v>
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
@@ -6388,7 +6388,7 @@
         </is>
       </c>
       <c r="E198" s="2" t="n">
-        <v>0.244</v>
+        <v>0.3</v>
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
@@ -6418,7 +6418,7 @@
         </is>
       </c>
       <c r="E199" s="2" t="n">
-        <v>0.217</v>
+        <v>0.234</v>
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
         </is>
       </c>
       <c r="E200" s="2" t="n">
-        <v>0.257</v>
+        <v>0.311</v>
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
@@ -6478,7 +6478,7 @@
         </is>
       </c>
       <c r="E201" s="2" t="n">
-        <v>0.217</v>
+        <v>0.265</v>
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="E202" s="2" t="n">
-        <v>0.286</v>
+        <v>0.305</v>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="E203" s="2" t="n">
-        <v>0.224</v>
+        <v>0.266</v>
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
@@ -6568,7 +6568,7 @@
         </is>
       </c>
       <c r="E204" s="2" t="n">
-        <v>0.273</v>
+        <v>0.299</v>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="E205" s="2" t="n">
-        <v>0.22</v>
+        <v>0.246</v>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
@@ -6628,7 +6628,7 @@
         </is>
       </c>
       <c r="E206" s="2" t="n">
-        <v>0.249</v>
+        <v>0.309</v>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
@@ -6658,7 +6658,7 @@
         </is>
       </c>
       <c r="E207" s="2" t="n">
-        <v>0.22</v>
+        <v>0.246</v>
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
@@ -6688,7 +6688,7 @@
         </is>
       </c>
       <c r="E208" s="2" t="n">
-        <v>0.258</v>
+        <v>0.3</v>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
@@ -6718,7 +6718,7 @@
         </is>
       </c>
       <c r="E209" s="2" t="n">
-        <v>0.219</v>
+        <v>0.278</v>
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
         </is>
       </c>
       <c r="E210" s="2" t="n">
-        <v>0.31</v>
+        <v>0.308</v>
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
@@ -6778,7 +6778,7 @@
         </is>
       </c>
       <c r="E211" s="2" t="n">
-        <v>0.231</v>
+        <v>0.25</v>
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="E212" s="2" t="n">
-        <v>3.164</v>
+        <v>3.579</v>
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
@@ -6838,7 +6838,7 @@
         </is>
       </c>
       <c r="E213" s="2" t="n">
-        <v>0.265</v>
+        <v>0.293</v>
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
@@ -6868,7 +6868,7 @@
         </is>
       </c>
       <c r="E214" s="2" t="n">
-        <v>0.25</v>
+        <v>0.303</v>
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         </is>
       </c>
       <c r="E215" s="2" t="n">
-        <v>0.221</v>
+        <v>0.287</v>
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
@@ -6928,7 +6928,7 @@
         </is>
       </c>
       <c r="E216" s="2" t="n">
-        <v>0.267</v>
+        <v>0.331</v>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
@@ -6958,7 +6958,7 @@
         </is>
       </c>
       <c r="E217" s="2" t="n">
-        <v>0.234</v>
+        <v>0.267</v>
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
@@ -6988,7 +6988,7 @@
         </is>
       </c>
       <c r="E218" s="2" t="n">
-        <v>0.117</v>
+        <v>0.257</v>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
@@ -7018,7 +7018,7 @@
         </is>
       </c>
       <c r="E219" s="2" t="n">
-        <v>0.316</v>
+        <v>0.337</v>
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
         </is>
       </c>
       <c r="E220" s="2" t="n">
-        <v>0.259</v>
+        <v>0.214</v>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
@@ -7078,7 +7078,7 @@
         </is>
       </c>
       <c r="E221" s="2" t="n">
-        <v>0.227</v>
+        <v>0.302</v>
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
@@ -7108,7 +7108,7 @@
         </is>
       </c>
       <c r="E222" s="2" t="n">
-        <v>0.29</v>
+        <v>0.293</v>
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
@@ -7138,7 +7138,7 @@
         </is>
       </c>
       <c r="E223" s="2" t="n">
-        <v>0.224</v>
+        <v>0.311</v>
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
@@ -7168,7 +7168,7 @@
         </is>
       </c>
       <c r="E224" s="2" t="n">
-        <v>0.233</v>
+        <v>0.319</v>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
         </is>
       </c>
       <c r="E225" s="2" t="n">
-        <v>0.251</v>
+        <v>0.268</v>
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
@@ -7228,7 +7228,7 @@
         </is>
       </c>
       <c r="E226" s="2" t="n">
-        <v>0.215</v>
+        <v>0.314</v>
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
@@ -7258,7 +7258,7 @@
         </is>
       </c>
       <c r="E227" s="2" t="n">
-        <v>0.239</v>
+        <v>0.306</v>
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
@@ -7288,7 +7288,7 @@
         </is>
       </c>
       <c r="E228" s="2" t="n">
-        <v>0.251</v>
+        <v>0.32</v>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
@@ -7318,7 +7318,7 @@
         </is>
       </c>
       <c r="E229" s="2" t="n">
-        <v>0.344</v>
+        <v>0.343</v>
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
         </is>
       </c>
       <c r="E230" s="2" t="n">
-        <v>0.234</v>
+        <v>0.325</v>
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
@@ -7378,7 +7378,7 @@
         </is>
       </c>
       <c r="E231" s="2" t="n">
-        <v>0.267</v>
+        <v>0.291</v>
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="E232" s="2" t="n">
-        <v>0.22</v>
+        <v>0.301</v>
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
@@ -7438,7 +7438,7 @@
         </is>
       </c>
       <c r="E233" s="2" t="n">
-        <v>0.237</v>
+        <v>0.335</v>
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
@@ -7468,7 +7468,7 @@
         </is>
       </c>
       <c r="E234" s="2" t="n">
-        <v>0.215</v>
+        <v>0.318</v>
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
         </is>
       </c>
       <c r="E235" s="2" t="n">
-        <v>0.261</v>
+        <v>0.309</v>
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
@@ -7528,7 +7528,7 @@
         </is>
       </c>
       <c r="E236" s="2" t="n">
-        <v>0.222</v>
+        <v>0.322</v>
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
@@ -7558,7 +7558,7 @@
         </is>
       </c>
       <c r="E237" s="2" t="n">
-        <v>0.277</v>
+        <v>0.322</v>
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
@@ -7588,7 +7588,7 @@
         </is>
       </c>
       <c r="E238" s="2" t="n">
-        <v>0.22</v>
+        <v>0.303</v>
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
@@ -7618,7 +7618,7 @@
         </is>
       </c>
       <c r="E239" s="2" t="n">
-        <v>0.133</v>
+        <v>0.369</v>
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         </is>
       </c>
       <c r="E240" s="2" t="n">
-        <v>0.363</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
@@ -7678,7 +7678,7 @@
         </is>
       </c>
       <c r="E241" s="2" t="n">
-        <v>0.253</v>
+        <v>0.294</v>
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="E242" s="2" t="n">
-        <v>0.226</v>
+        <v>0.292</v>
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
@@ -7738,7 +7738,7 @@
         </is>
       </c>
       <c r="E243" s="2" t="n">
-        <v>0.126</v>
+        <v>0.285</v>
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
@@ -7768,7 +7768,7 @@
         </is>
       </c>
       <c r="E244" s="2" t="n">
-        <v>0.285</v>
+        <v>0.284</v>
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
         </is>
       </c>
       <c r="E245" s="2" t="n">
-        <v>0.26</v>
+        <v>0.291</v>
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
@@ -7828,7 +7828,7 @@
         </is>
       </c>
       <c r="E246" s="2" t="n">
-        <v>0.235</v>
+        <v>0.292</v>
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
         </is>
       </c>
       <c r="E247" s="2" t="n">
-        <v>0.249</v>
+        <v>0.284</v>
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
@@ -7888,7 +7888,7 @@
         </is>
       </c>
       <c r="E248" s="2" t="n">
-        <v>0.213</v>
+        <v>0.282</v>
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
@@ -7918,7 +7918,7 @@
         </is>
       </c>
       <c r="E249" s="2" t="n">
-        <v>0.2</v>
+        <v>0.283</v>
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
@@ -7948,7 +7948,7 @@
         </is>
       </c>
       <c r="E250" s="2" t="n">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
@@ -7978,7 +7978,7 @@
         </is>
       </c>
       <c r="E251" s="2" t="n">
-        <v>0.246</v>
+        <v>0.305</v>
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
         </is>
       </c>
       <c r="E252" s="2" t="n">
-        <v>0.216</v>
+        <v>0.296</v>
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
@@ -8038,7 +8038,7 @@
         </is>
       </c>
       <c r="E253" s="2" t="n">
-        <v>0.281</v>
+        <v>0.286</v>
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
@@ -8068,7 +8068,7 @@
         </is>
       </c>
       <c r="E254" s="2" t="n">
-        <v>0.255</v>
+        <v>0.228</v>
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
         </is>
       </c>
       <c r="E255" s="2" t="n">
-        <v>0.257</v>
+        <v>0.313</v>
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
@@ -8128,7 +8128,7 @@
         </is>
       </c>
       <c r="E256" s="2" t="n">
-        <v>0.246</v>
+        <v>0.257</v>
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="E257" s="2" t="n">
-        <v>0.256</v>
+        <v>0.307</v>
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
@@ -8188,7 +8188,7 @@
         </is>
       </c>
       <c r="E258" s="2" t="n">
-        <v>0.227</v>
+        <v>0.293</v>
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
@@ -8218,7 +8218,7 @@
         </is>
       </c>
       <c r="E259" s="2" t="n">
-        <v>0.198</v>
+        <v>0.257</v>
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
@@ -8248,7 +8248,7 @@
         </is>
       </c>
       <c r="E260" s="2" t="n">
-        <v>0.233</v>
+        <v>0.299</v>
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
@@ -8278,7 +8278,7 @@
         </is>
       </c>
       <c r="E261" s="2" t="n">
-        <v>0.226</v>
+        <v>0.282</v>
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="E262" s="2" t="n">
-        <v>3.259</v>
+        <v>2.493</v>
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
@@ -8338,7 +8338,7 @@
         </is>
       </c>
       <c r="E263" s="2" t="n">
-        <v>0.268</v>
+        <v>0.303</v>
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
@@ -8368,7 +8368,7 @@
         </is>
       </c>
       <c r="E264" s="2" t="n">
-        <v>0.307</v>
+        <v>0.291</v>
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
@@ -8398,7 +8398,7 @@
         </is>
       </c>
       <c r="E265" s="2" t="n">
-        <v>0.216</v>
+        <v>0.314</v>
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
@@ -8428,7 +8428,7 @@
         </is>
       </c>
       <c r="E266" s="2" t="n">
-        <v>0.263</v>
+        <v>0.266</v>
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
@@ -8458,7 +8458,7 @@
         </is>
       </c>
       <c r="E267" s="2" t="n">
-        <v>0.222</v>
+        <v>0.284</v>
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="E268" s="2" t="n">
-        <v>0.286</v>
+        <v>0.424</v>
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
@@ -8518,7 +8518,7 @@
         </is>
       </c>
       <c r="E269" s="2" t="n">
-        <v>0.229</v>
+        <v>0.25</v>
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
@@ -8548,7 +8548,7 @@
         </is>
       </c>
       <c r="E270" s="2" t="n">
-        <v>0.269</v>
+        <v>0.376</v>
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         </is>
       </c>
       <c r="E271" s="2" t="n">
-        <v>0.224</v>
+        <v>0.274</v>
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="E272" s="2" t="n">
-        <v>0.257</v>
+        <v>0.364</v>
       </c>
       <c r="F272" s="2" t="inlineStr">
         <is>
@@ -8638,7 +8638,7 @@
         </is>
       </c>
       <c r="E273" s="2" t="n">
-        <v>0.219</v>
+        <v>0.317</v>
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
@@ -8668,7 +8668,7 @@
         </is>
       </c>
       <c r="E274" s="2" t="n">
-        <v>0.257</v>
+        <v>0.258</v>
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
         </is>
       </c>
       <c r="E275" s="2" t="n">
-        <v>0.222</v>
+        <v>0.297</v>
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
@@ -8728,7 +8728,7 @@
         </is>
       </c>
       <c r="E276" s="2" t="n">
-        <v>0.28</v>
+        <v>0.272</v>
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
@@ -8758,7 +8758,7 @@
         </is>
       </c>
       <c r="E277" s="2" t="n">
-        <v>0.219</v>
+        <v>0.25</v>
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="E278" s="2" t="n">
-        <v>0.29</v>
+        <v>0.292</v>
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
@@ -8818,7 +8818,7 @@
         </is>
       </c>
       <c r="E279" s="2" t="n">
-        <v>0.222</v>
+        <v>0.272</v>
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
@@ -8848,7 +8848,7 @@
         </is>
       </c>
       <c r="E280" s="2" t="n">
-        <v>0.251</v>
+        <v>0.249</v>
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
@@ -8878,7 +8878,7 @@
         </is>
       </c>
       <c r="E281" s="2" t="n">
-        <v>0.217</v>
+        <v>0.313</v>
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
@@ -8908,7 +8908,7 @@
         </is>
       </c>
       <c r="E282" s="2" t="n">
-        <v>0.255</v>
+        <v>0.275</v>
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
@@ -8938,7 +8938,7 @@
         </is>
       </c>
       <c r="E283" s="2" t="n">
-        <v>0.218</v>
+        <v>0.248</v>
       </c>
       <c r="F283" s="2" t="inlineStr">
         <is>
@@ -8968,7 +8968,7 @@
         </is>
       </c>
       <c r="E284" s="2" t="n">
-        <v>0.271</v>
+        <v>0.298</v>
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
         </is>
       </c>
       <c r="E285" s="2" t="n">
-        <v>0.201</v>
+        <v>0.334</v>
       </c>
       <c r="F285" s="2" t="inlineStr">
         <is>
@@ -9028,7 +9028,7 @@
         </is>
       </c>
       <c r="E286" s="2" t="n">
-        <v>0.263</v>
+        <v>0.309</v>
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="E287" s="2" t="n">
-        <v>0.219</v>
+        <v>0.316</v>
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
@@ -9088,7 +9088,7 @@
         </is>
       </c>
       <c r="E288" s="2" t="n">
-        <v>0.199</v>
+        <v>0.293</v>
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
@@ -9118,7 +9118,7 @@
         </is>
       </c>
       <c r="E289" s="2" t="n">
-        <v>0.252</v>
+        <v>0.269</v>
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
         </is>
       </c>
       <c r="E290" s="2" t="n">
-        <v>0.217</v>
+        <v>0.3</v>
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
@@ -9178,7 +9178,7 @@
         </is>
       </c>
       <c r="E291" s="2" t="n">
-        <v>0.217</v>
+        <v>0.274</v>
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
@@ -9208,7 +9208,7 @@
         </is>
       </c>
       <c r="E292" s="2" t="n">
-        <v>0.26</v>
+        <v>0.255</v>
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
@@ -9238,7 +9238,7 @@
         </is>
       </c>
       <c r="E293" s="2" t="n">
-        <v>0.213</v>
+        <v>0.342</v>
       </c>
       <c r="F293" s="2" t="inlineStr">
         <is>
@@ -9268,7 +9268,7 @@
         </is>
       </c>
       <c r="E294" s="2" t="n">
-        <v>0.263</v>
+        <v>0.305</v>
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
         </is>
       </c>
       <c r="E295" s="2" t="n">
-        <v>0.223</v>
+        <v>0.3</v>
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
@@ -9328,7 +9328,7 @@
         </is>
       </c>
       <c r="E296" s="2" t="n">
-        <v>0.288</v>
+        <v>0.303</v>
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
         </is>
       </c>
       <c r="E297" s="2" t="n">
-        <v>0.282</v>
+        <v>0.296</v>
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
@@ -9388,7 +9388,7 @@
         </is>
       </c>
       <c r="E298" s="2" t="n">
-        <v>0.238</v>
+        <v>0.307</v>
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
@@ -9418,7 +9418,7 @@
         </is>
       </c>
       <c r="E299" s="2" t="n">
-        <v>0.215</v>
+        <v>0.298</v>
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
         </is>
       </c>
       <c r="E300" s="2" t="n">
-        <v>0.258</v>
+        <v>0.318</v>
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
@@ -9478,7 +9478,7 @@
         </is>
       </c>
       <c r="E301" s="2" t="n">
-        <v>0.195</v>
+        <v>0.265</v>
       </c>
       <c r="F301" s="2" t="inlineStr">
         <is>
@@ -9508,7 +9508,7 @@
         </is>
       </c>
       <c r="E302" s="2" t="n">
-        <v>1.322</v>
+        <v>2.101</v>
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
@@ -9538,7 +9538,7 @@
         </is>
       </c>
       <c r="E303" s="2" t="n">
-        <v>0.261</v>
+        <v>0.294</v>
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
@@ -9568,7 +9568,7 @@
         </is>
       </c>
       <c r="E304" s="2" t="n">
-        <v>0.277</v>
+        <v>0.308</v>
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
@@ -9598,7 +9598,7 @@
         </is>
       </c>
       <c r="E305" s="2" t="n">
-        <v>0.217</v>
+        <v>0.268</v>
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="E306" s="2" t="n">
-        <v>0.257</v>
+        <v>0.254</v>
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
@@ -9658,7 +9658,7 @@
         </is>
       </c>
       <c r="E307" s="2" t="n">
-        <v>0.198</v>
+        <v>0.293</v>
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
@@ -9688,7 +9688,7 @@
         </is>
       </c>
       <c r="E308" s="2" t="n">
-        <v>0.26</v>
+        <v>0.291</v>
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
@@ -9718,7 +9718,7 @@
         </is>
       </c>
       <c r="E309" s="2" t="n">
-        <v>0.231</v>
+        <v>0.25</v>
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
@@ -9748,7 +9748,7 @@
         </is>
       </c>
       <c r="E310" s="2" t="n">
-        <v>0.285</v>
+        <v>0.289</v>
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
         </is>
       </c>
       <c r="E311" s="2" t="n">
-        <v>0.242</v>
+        <v>0.275</v>
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
@@ -9808,7 +9808,7 @@
         </is>
       </c>
       <c r="E312" s="2" t="n">
-        <v>0.24</v>
+        <v>0.254</v>
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
@@ -9838,7 +9838,7 @@
         </is>
       </c>
       <c r="E313" s="2" t="n">
-        <v>0.27</v>
+        <v>0.314</v>
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
@@ -9868,7 +9868,7 @@
         </is>
       </c>
       <c r="E314" s="2" t="n">
-        <v>0.22</v>
+        <v>0.257</v>
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
         </is>
       </c>
       <c r="E315" s="2" t="n">
-        <v>0.273</v>
+        <v>0.297</v>
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
@@ -9928,7 +9928,7 @@
         </is>
       </c>
       <c r="E316" s="2" t="n">
-        <v>0.235</v>
+        <v>0.291</v>
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
@@ -9958,7 +9958,7 @@
         </is>
       </c>
       <c r="E317" s="2" t="n">
-        <v>0.262</v>
+        <v>0.239</v>
       </c>
       <c r="F317" s="2" t="inlineStr">
         <is>
@@ -9988,7 +9988,7 @@
         </is>
       </c>
       <c r="E318" s="2" t="n">
-        <v>0.216</v>
+        <v>0.293</v>
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="E319" s="2" t="n">
-        <v>0.346</v>
+        <v>0.272</v>
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
         </is>
       </c>
       <c r="E320" s="2" t="n">
-        <v>0.226</v>
+        <v>0.264</v>
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
@@ -10078,7 +10078,7 @@
         </is>
       </c>
       <c r="E321" s="2" t="n">
-        <v>0.256</v>
+        <v>0.292</v>
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
@@ -10108,7 +10108,7 @@
         </is>
       </c>
       <c r="E322" s="2" t="n">
-        <v>5.883</v>
+        <v>4.026</v>
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
@@ -10138,7 +10138,7 @@
         </is>
       </c>
       <c r="E323" s="2" t="n">
-        <v>0.215</v>
+        <v>0.28</v>
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
@@ -10168,7 +10168,7 @@
         </is>
       </c>
       <c r="E324" s="2" t="n">
-        <v>0.268</v>
+        <v>0.276</v>
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="E325" s="2" t="n">
-        <v>0.219</v>
+        <v>0.278</v>
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="E326" s="2" t="n">
-        <v>0.264</v>
+        <v>0.31</v>
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
@@ -10258,7 +10258,7 @@
         </is>
       </c>
       <c r="E327" s="2" t="n">
-        <v>0.219</v>
+        <v>0.269</v>
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
@@ -10288,7 +10288,7 @@
         </is>
       </c>
       <c r="E328" s="2" t="n">
-        <v>0.27</v>
+        <v>0.249</v>
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
@@ -10318,7 +10318,7 @@
         </is>
       </c>
       <c r="E329" s="2" t="n">
-        <v>0.214</v>
+        <v>0.309</v>
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
@@ -10348,7 +10348,7 @@
         </is>
       </c>
       <c r="E330" s="2" t="n">
-        <v>0.249</v>
+        <v>0.275</v>
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
@@ -10378,7 +10378,7 @@
         </is>
       </c>
       <c r="E331" s="2" t="n">
-        <v>0.217</v>
+        <v>0.251</v>
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="E332" s="2" t="n">
-        <v>0.211</v>
+        <v>0.292</v>
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="E333" s="2" t="n">
-        <v>0.289</v>
+        <v>0.259</v>
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="E334" s="2" t="n">
-        <v>0.208</v>
+        <v>0.285</v>
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
         </is>
       </c>
       <c r="E335" s="2" t="n">
-        <v>0.11</v>
+        <v>0.291</v>
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
@@ -10528,7 +10528,7 @@
         </is>
       </c>
       <c r="E336" s="2" t="n">
-        <v>0.255</v>
+        <v>0.285</v>
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
@@ -10558,7 +10558,7 @@
         </is>
       </c>
       <c r="E337" s="2" t="n">
-        <v>0.275</v>
+        <v>0.28</v>
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
@@ -10588,7 +10588,7 @@
         </is>
       </c>
       <c r="E338" s="2" t="n">
-        <v>0.199</v>
+        <v>0.279</v>
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
@@ -10618,7 +10618,7 @@
         </is>
       </c>
       <c r="E339" s="2" t="n">
-        <v>0.264</v>
+        <v>0.283</v>
       </c>
       <c r="F339" s="2" t="inlineStr">
         <is>
@@ -10648,7 +10648,7 @@
         </is>
       </c>
       <c r="E340" s="2" t="n">
-        <v>0.221</v>
+        <v>0.281</v>
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="E341" s="2" t="n">
-        <v>0.262</v>
+        <v>0.288</v>
       </c>
       <c r="F341" s="2" t="inlineStr">
         <is>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="E342" s="2" t="n">
-        <v>2.034</v>
+        <v>2.717</v>
       </c>
       <c r="F342" s="2" t="inlineStr">
         <is>
@@ -10738,7 +10738,7 @@
         </is>
       </c>
       <c r="E343" s="2" t="n">
-        <v>0.216</v>
+        <v>0.254</v>
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
@@ -10768,7 +10768,7 @@
         </is>
       </c>
       <c r="E344" s="2" t="n">
-        <v>0.263</v>
+        <v>0.282</v>
       </c>
       <c r="F344" s="2" t="inlineStr">
         <is>
@@ -10798,7 +10798,7 @@
         </is>
       </c>
       <c r="E345" s="2" t="n">
-        <v>0.22</v>
+        <v>0.253</v>
       </c>
       <c r="F345" s="2" t="inlineStr">
         <is>
@@ -10828,7 +10828,7 @@
         </is>
       </c>
       <c r="E346" s="2" t="n">
-        <v>0.249</v>
+        <v>0.335</v>
       </c>
       <c r="F346" s="2" t="inlineStr">
         <is>
@@ -10858,7 +10858,7 @@
         </is>
       </c>
       <c r="E347" s="2" t="n">
-        <v>0.223</v>
+        <v>0.26</v>
       </c>
       <c r="F347" s="2" t="inlineStr">
         <is>
@@ -10888,7 +10888,7 @@
         </is>
       </c>
       <c r="E348" s="2" t="n">
-        <v>0.198</v>
+        <v>0.335</v>
       </c>
       <c r="F348" s="2" t="inlineStr">
         <is>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="E349" s="2" t="n">
-        <v>0.26</v>
+        <v>0.222</v>
       </c>
       <c r="F349" s="2" t="inlineStr">
         <is>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="E350" s="2" t="n">
-        <v>0.216</v>
+        <v>0.293</v>
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
@@ -10978,7 +10978,7 @@
         </is>
       </c>
       <c r="E351" s="2" t="n">
-        <v>0.278</v>
+        <v>0.318</v>
       </c>
       <c r="F351" s="2" t="inlineStr">
         <is>
@@ -11008,7 +11008,7 @@
         </is>
       </c>
       <c r="E352" s="2" t="n">
-        <v>0.213</v>
+        <v>0.284</v>
       </c>
       <c r="F352" s="2" t="inlineStr">
         <is>
@@ -11038,7 +11038,7 @@
         </is>
       </c>
       <c r="E353" s="2" t="n">
-        <v>0.251</v>
+        <v>0.255</v>
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
@@ -11068,7 +11068,7 @@
         </is>
       </c>
       <c r="E354" s="2" t="n">
-        <v>0.226</v>
+        <v>0.296</v>
       </c>
       <c r="F354" s="2" t="inlineStr">
         <is>
@@ -11098,7 +11098,7 @@
         </is>
       </c>
       <c r="E355" s="2" t="n">
-        <v>0.25</v>
+        <v>0.264</v>
       </c>
       <c r="F355" s="2" t="inlineStr">
         <is>
@@ -11128,7 +11128,7 @@
         </is>
       </c>
       <c r="E356" s="2" t="n">
-        <v>0.241</v>
+        <v>0.254</v>
       </c>
       <c r="F356" s="2" t="inlineStr">
         <is>
@@ -11158,7 +11158,7 @@
         </is>
       </c>
       <c r="E357" s="2" t="n">
-        <v>0.261</v>
+        <v>0.3</v>
       </c>
       <c r="F357" s="2" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
         </is>
       </c>
       <c r="E358" s="2" t="n">
-        <v>0.21</v>
+        <v>0.263</v>
       </c>
       <c r="F358" s="2" t="inlineStr">
         <is>
@@ -11218,7 +11218,7 @@
         </is>
       </c>
       <c r="E359" s="2" t="n">
-        <v>0.254</v>
+        <v>0.246</v>
       </c>
       <c r="F359" s="2" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
         </is>
       </c>
       <c r="E360" s="2" t="n">
-        <v>0.211</v>
+        <v>0.288</v>
       </c>
       <c r="F360" s="2" t="inlineStr">
         <is>
@@ -11278,7 +11278,7 @@
         </is>
       </c>
       <c r="E361" s="2" t="n">
-        <v>0.243</v>
+        <v>0.283</v>
       </c>
       <c r="F361" s="2" t="inlineStr">
         <is>
@@ -11308,7 +11308,7 @@
         </is>
       </c>
       <c r="E362" s="2" t="n">
-        <v>9.519</v>
+        <v>2.206</v>
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
@@ -11338,7 +11338,7 @@
         </is>
       </c>
       <c r="E363" s="2" t="n">
-        <v>0.283</v>
+        <v>0.295</v>
       </c>
       <c r="F363" s="2" t="inlineStr">
         <is>
@@ -11368,7 +11368,7 @@
         </is>
       </c>
       <c r="E364" s="2" t="n">
-        <v>0.23</v>
+        <v>0.288</v>
       </c>
       <c r="F364" s="2" t="inlineStr">
         <is>
@@ -11398,7 +11398,7 @@
         </is>
       </c>
       <c r="E365" s="2" t="n">
-        <v>0.224</v>
+        <v>0.343</v>
       </c>
       <c r="F365" s="2" t="inlineStr">
         <is>
@@ -11428,7 +11428,7 @@
         </is>
       </c>
       <c r="E366" s="2" t="n">
-        <v>0.257</v>
+        <v>0.251</v>
       </c>
       <c r="F366" s="2" t="inlineStr">
         <is>
@@ -11458,7 +11458,7 @@
         </is>
       </c>
       <c r="E367" s="2" t="n">
-        <v>0.223</v>
+        <v>0.32</v>
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
@@ -11488,7 +11488,7 @@
         </is>
       </c>
       <c r="E368" s="2" t="n">
-        <v>0.252</v>
+        <v>0.257</v>
       </c>
       <c r="F368" s="2" t="inlineStr">
         <is>
@@ -11518,7 +11518,7 @@
         </is>
       </c>
       <c r="E369" s="2" t="n">
-        <v>0.222</v>
+        <v>0.309</v>
       </c>
       <c r="F369" s="2" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
       <c r="E370" s="2" t="n">
-        <v>0.214</v>
+        <v>0.251</v>
       </c>
       <c r="F370" s="2" t="inlineStr">
         <is>
@@ -11578,7 +11578,7 @@
         </is>
       </c>
       <c r="E371" s="2" t="n">
-        <v>0.268</v>
+        <v>0.294</v>
       </c>
       <c r="F371" s="2" t="inlineStr">
         <is>
@@ -11608,7 +11608,7 @@
         </is>
       </c>
       <c r="E372" s="2" t="n">
-        <v>0.227</v>
+        <v>0.324</v>
       </c>
       <c r="F372" s="2" t="inlineStr">
         <is>
@@ -11638,7 +11638,7 @@
         </is>
       </c>
       <c r="E373" s="2" t="n">
-        <v>0.262</v>
+        <v>0.266</v>
       </c>
       <c r="F373" s="2" t="inlineStr">
         <is>
@@ -11668,7 +11668,7 @@
         </is>
       </c>
       <c r="E374" s="2" t="n">
-        <v>0.222</v>
+        <v>0.252</v>
       </c>
       <c r="F374" s="2" t="inlineStr">
         <is>
@@ -11698,7 +11698,7 @@
         </is>
       </c>
       <c r="E375" s="2" t="n">
-        <v>0.22</v>
+        <v>0.309</v>
       </c>
       <c r="F375" s="2" t="inlineStr">
         <is>
@@ -11728,7 +11728,7 @@
         </is>
       </c>
       <c r="E376" s="2" t="n">
-        <v>0.267</v>
+        <v>0.252</v>
       </c>
       <c r="F376" s="2" t="inlineStr">
         <is>
@@ -11758,7 +11758,7 @@
         </is>
       </c>
       <c r="E377" s="2" t="n">
-        <v>0.217</v>
+        <v>0.287</v>
       </c>
       <c r="F377" s="2" t="inlineStr">
         <is>
@@ -11788,7 +11788,7 @@
         </is>
       </c>
       <c r="E378" s="2" t="n">
-        <v>0.259</v>
+        <v>0.311</v>
       </c>
       <c r="F378" s="2" t="inlineStr">
         <is>
@@ -11818,7 +11818,7 @@
         </is>
       </c>
       <c r="E379" s="2" t="n">
-        <v>0.213</v>
+        <v>0.264</v>
       </c>
       <c r="F379" s="2" t="inlineStr">
         <is>
@@ -11848,7 +11848,7 @@
         </is>
       </c>
       <c r="E380" s="2" t="n">
-        <v>0.254</v>
+        <v>0.246</v>
       </c>
       <c r="F380" s="2" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
         </is>
       </c>
       <c r="E381" s="2" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="F381" s="2" t="inlineStr">
         <is>
@@ -11908,7 +11908,7 @@
         </is>
       </c>
       <c r="E382" s="2" t="n">
-        <v>13.297</v>
+        <v>2.437</v>
       </c>
       <c r="F382" s="2" t="inlineStr">
         <is>
@@ -11938,7 +11938,7 @@
         </is>
       </c>
       <c r="E383" s="2" t="n">
-        <v>0.292</v>
+        <v>0.272</v>
       </c>
       <c r="F383" s="2" t="inlineStr">
         <is>
@@ -11968,7 +11968,7 @@
         </is>
       </c>
       <c r="E384" s="2" t="n">
-        <v>0.245</v>
+        <v>0.292</v>
       </c>
       <c r="F384" s="2" t="inlineStr">
         <is>
@@ -11998,7 +11998,7 @@
         </is>
       </c>
       <c r="E385" s="2" t="n">
-        <v>0.281</v>
+        <v>0.267</v>
       </c>
       <c r="F385" s="2" t="inlineStr">
         <is>
@@ -12028,7 +12028,7 @@
         </is>
       </c>
       <c r="E386" s="2" t="n">
-        <v>0.472</v>
+        <v>0.667</v>
       </c>
       <c r="F386" s="2" t="inlineStr">
         <is>
@@ -12058,7 +12058,7 @@
         </is>
       </c>
       <c r="E387" s="2" t="n">
-        <v>0.388</v>
+        <v>0.274</v>
       </c>
       <c r="F387" s="2" t="inlineStr">
         <is>
@@ -12088,7 +12088,7 @@
         </is>
       </c>
       <c r="E388" s="2" t="n">
-        <v>0.283</v>
+        <v>0.303</v>
       </c>
       <c r="F388" s="2" t="inlineStr">
         <is>
@@ -12118,7 +12118,7 @@
         </is>
       </c>
       <c r="E389" s="2" t="n">
-        <v>0.266</v>
+        <v>0.332</v>
       </c>
       <c r="F389" s="2" t="inlineStr">
         <is>
@@ -12148,7 +12148,7 @@
         </is>
       </c>
       <c r="E390" s="2" t="n">
-        <v>0.588</v>
+        <v>0.653</v>
       </c>
       <c r="F390" s="2" t="inlineStr">
         <is>
@@ -12178,7 +12178,7 @@
         </is>
       </c>
       <c r="E391" s="2" t="n">
-        <v>0.252</v>
+        <v>0.272</v>
       </c>
       <c r="F391" s="2" t="inlineStr">
         <is>
@@ -12208,7 +12208,7 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>0.304</v>
+        <v>0.336</v>
       </c>
       <c r="F392" s="2" t="inlineStr">
         <is>
@@ -12238,7 +12238,7 @@
         </is>
       </c>
       <c r="E393" s="2" t="n">
-        <v>0.239</v>
+        <v>0.271</v>
       </c>
       <c r="F393" s="2" t="inlineStr">
         <is>
@@ -12268,7 +12268,7 @@
         </is>
       </c>
       <c r="E394" s="2" t="n">
-        <v>0.622</v>
+        <v>0.656</v>
       </c>
       <c r="F394" s="2" t="inlineStr">
         <is>
@@ -12298,7 +12298,7 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>0.246</v>
+        <v>0.296</v>
       </c>
       <c r="F395" s="2" t="inlineStr">
         <is>
@@ -12328,7 +12328,7 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>0.274</v>
+        <v>0.284</v>
       </c>
       <c r="F396" s="2" t="inlineStr">
         <is>
@@ -12358,7 +12358,7 @@
         </is>
       </c>
       <c r="E397" s="2" t="n">
-        <v>0.248</v>
+        <v>0.312</v>
       </c>
       <c r="F397" s="2" t="inlineStr">
         <is>
@@ -12388,7 +12388,7 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.623</v>
       </c>
       <c r="F398" s="2" t="inlineStr">
         <is>
@@ -12418,7 +12418,7 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>0.285</v>
+        <v>0.28</v>
       </c>
       <c r="F399" s="2" t="inlineStr">
         <is>
@@ -12448,7 +12448,7 @@
         </is>
       </c>
       <c r="E400" s="2" t="n">
-        <v>0.229</v>
+        <v>0.308</v>
       </c>
       <c r="F400" s="2" t="inlineStr">
         <is>
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="E401" s="2" t="n">
-        <v>0.302</v>
+        <v>0.24</v>
       </c>
       <c r="F401" s="2" t="inlineStr">
         <is>
@@ -12508,7 +12508,7 @@
         </is>
       </c>
       <c r="E402" s="2" t="n">
-        <v>14.691</v>
+        <v>1.922</v>
       </c>
       <c r="F402" s="2" t="inlineStr">
         <is>
@@ -12538,7 +12538,7 @@
         </is>
       </c>
       <c r="E403" s="2" t="n">
-        <v>0.176</v>
+        <v>0.178</v>
       </c>
       <c r="F403" s="2" t="inlineStr">
         <is>
@@ -12568,7 +12568,7 @@
         </is>
       </c>
       <c r="E404" s="2" t="n">
-        <v>0.125</v>
+        <v>0.211</v>
       </c>
       <c r="F404" s="2" t="inlineStr">
         <is>
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="E405" s="2" t="n">
-        <v>0.158</v>
+        <v>0.181</v>
       </c>
       <c r="F405" s="2" t="inlineStr">
         <is>
@@ -12628,7 +12628,7 @@
         </is>
       </c>
       <c r="E406" s="2" t="n">
-        <v>0.115</v>
+        <v>0.16</v>
       </c>
       <c r="F406" s="2" t="inlineStr">
         <is>
@@ -12658,7 +12658,7 @@
         </is>
       </c>
       <c r="E407" s="2" t="n">
-        <v>0.174</v>
+        <v>0.2</v>
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
@@ -12688,7 +12688,7 @@
         </is>
       </c>
       <c r="E408" s="2" t="n">
-        <v>0.119</v>
+        <v>0.205</v>
       </c>
       <c r="F408" s="2" t="inlineStr">
         <is>
@@ -12718,7 +12718,7 @@
         </is>
       </c>
       <c r="E409" s="2" t="n">
-        <v>0.108</v>
+        <v>0.17</v>
       </c>
       <c r="F409" s="2" t="inlineStr">
         <is>
@@ -12748,7 +12748,7 @@
         </is>
       </c>
       <c r="E410" s="2" t="n">
-        <v>0.168</v>
+        <v>0.23</v>
       </c>
       <c r="F410" s="2" t="inlineStr">
         <is>
@@ -12778,7 +12778,7 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>0.13</v>
+        <v>0.161</v>
       </c>
       <c r="F411" s="2" t="inlineStr">
         <is>
@@ -12808,7 +12808,7 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>0.126</v>
+        <v>0.231</v>
       </c>
       <c r="F412" s="2" t="inlineStr">
         <is>
@@ -12838,7 +12838,7 @@
         </is>
       </c>
       <c r="E413" s="2" t="n">
-        <v>0.177</v>
+        <v>0.157</v>
       </c>
       <c r="F413" s="2" t="inlineStr">
         <is>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>0.121</v>
+        <v>0.2</v>
       </c>
       <c r="F414" s="2" t="inlineStr">
         <is>
@@ -12898,7 +12898,7 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>0.156</v>
+        <v>0.191</v>
       </c>
       <c r="F415" s="2" t="inlineStr">
         <is>
@@ -12928,7 +12928,7 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>0.117</v>
+        <v>0.188</v>
       </c>
       <c r="F416" s="2" t="inlineStr">
         <is>
@@ -12958,7 +12958,7 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>0.168</v>
+        <v>0.193</v>
       </c>
       <c r="F417" s="2" t="inlineStr">
         <is>
@@ -12988,7 +12988,7 @@
         </is>
       </c>
       <c r="E418" s="2" t="n">
-        <v>0.115</v>
+        <v>0.19</v>
       </c>
       <c r="F418" s="2" t="inlineStr">
         <is>
@@ -13018,7 +13018,7 @@
         </is>
       </c>
       <c r="E419" s="2" t="n">
-        <v>0.173</v>
+        <v>0.188</v>
       </c>
       <c r="F419" s="2" t="inlineStr">
         <is>
@@ -13048,7 +13048,7 @@
         </is>
       </c>
       <c r="E420" s="2" t="n">
-        <v>0.155</v>
+        <v>0.208</v>
       </c>
       <c r="F420" s="2" t="inlineStr">
         <is>
@@ -13078,7 +13078,7 @@
         </is>
       </c>
       <c r="E421" s="2" t="n">
-        <v>0.184</v>
+        <v>0.19</v>
       </c>
       <c r="F421" s="2" t="inlineStr">
         <is>
@@ -13108,7 +13108,7 @@
         </is>
       </c>
       <c r="E422" s="2" t="n">
-        <v>11.503</v>
+        <v>3.379</v>
       </c>
       <c r="F422" s="2" t="inlineStr">
         <is>
@@ -13138,7 +13138,7 @@
         </is>
       </c>
       <c r="E423" s="2" t="n">
-        <v>0.218</v>
+        <v>0.184</v>
       </c>
       <c r="F423" s="2" t="inlineStr">
         <is>
@@ -13168,7 +13168,7 @@
         </is>
       </c>
       <c r="E424" s="2" t="n">
-        <v>0.184</v>
+        <v>0.224</v>
       </c>
       <c r="F424" s="2" t="inlineStr">
         <is>
@@ -13198,7 +13198,7 @@
         </is>
       </c>
       <c r="E425" s="2" t="n">
-        <v>0.165</v>
+        <v>0.197</v>
       </c>
       <c r="F425" s="2" t="inlineStr">
         <is>
@@ -13228,7 +13228,7 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>0.21</v>
+        <v>0.254</v>
       </c>
       <c r="F426" s="2" t="inlineStr">
         <is>
@@ -13258,7 +13258,7 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>0.168</v>
+        <v>0.198</v>
       </c>
       <c r="F427" s="2" t="inlineStr">
         <is>
@@ -13288,7 +13288,7 @@
         </is>
       </c>
       <c r="E428" s="2" t="n">
-        <v>0.213</v>
+        <v>0.241</v>
       </c>
       <c r="F428" s="2" t="inlineStr">
         <is>
@@ -13318,7 +13318,7 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>0.168</v>
+        <v>0.27</v>
       </c>
       <c r="F429" s="2" t="inlineStr">
         <is>
@@ -13348,7 +13348,7 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>0.212</v>
+        <v>0.22</v>
       </c>
       <c r="F430" s="2" t="inlineStr">
         <is>
@@ -13378,7 +13378,7 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>0.173</v>
+        <v>0.201</v>
       </c>
       <c r="F431" s="2" t="inlineStr">
         <is>
@@ -13408,7 +13408,7 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>0.164</v>
+        <v>0.253</v>
       </c>
       <c r="F432" s="2" t="inlineStr">
         <is>
@@ -13438,7 +13438,7 @@
         </is>
       </c>
       <c r="E433" s="2" t="n">
-        <v>0.206</v>
+        <v>0.169</v>
       </c>
       <c r="F433" s="2" t="inlineStr">
         <is>
@@ -13468,7 +13468,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>0.178</v>
+        <v>0.236</v>
       </c>
       <c r="F434" s="2" t="inlineStr">
         <is>
@@ -13498,7 +13498,7 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>0.198</v>
+        <v>0.231</v>
       </c>
       <c r="F435" s="2" t="inlineStr">
         <is>
@@ -13528,7 +13528,7 @@
         </is>
       </c>
       <c r="E436" s="2" t="n">
-        <v>0.167</v>
+        <v>0.198</v>
       </c>
       <c r="F436" s="2" t="inlineStr">
         <is>
@@ -13558,7 +13558,7 @@
         </is>
       </c>
       <c r="E437" s="2" t="n">
-        <v>0.211</v>
+        <v>0.233</v>
       </c>
       <c r="F437" s="2" t="inlineStr">
         <is>
@@ -13588,7 +13588,7 @@
         </is>
       </c>
       <c r="E438" s="2" t="n">
-        <v>0.18</v>
+        <v>0.225</v>
       </c>
       <c r="F438" s="2" t="inlineStr">
         <is>
@@ -13618,7 +13618,7 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>0.164</v>
+        <v>0.213</v>
       </c>
       <c r="F439" s="2" t="inlineStr">
         <is>
@@ -13648,7 +13648,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>0.21</v>
+        <v>0.236</v>
       </c>
       <c r="F440" s="2" t="inlineStr">
         <is>
@@ -13678,7 +13678,7 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>0.17</v>
+        <v>0.219</v>
       </c>
       <c r="F441" s="2" t="inlineStr">
         <is>
@@ -13708,7 +13708,7 @@
         </is>
       </c>
       <c r="E442" s="2" t="n">
-        <v>0.217</v>
+        <v>0.198</v>
       </c>
       <c r="F442" s="2" t="inlineStr">
         <is>
@@ -13738,7 +13738,7 @@
         </is>
       </c>
       <c r="E443" s="2" t="n">
-        <v>0.182</v>
+        <v>0.256</v>
       </c>
       <c r="F443" s="2" t="inlineStr">
         <is>
@@ -13768,7 +13768,7 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>0.237</v>
+        <v>0.208</v>
       </c>
       <c r="F444" s="2" t="inlineStr">
         <is>
@@ -13798,7 +13798,7 @@
         </is>
       </c>
       <c r="E445" s="2" t="n">
-        <v>0.201</v>
+        <v>0.248</v>
       </c>
       <c r="F445" s="2" t="inlineStr">
         <is>
@@ -13828,7 +13828,7 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>0.167</v>
+        <v>0.174</v>
       </c>
       <c r="F446" s="2" t="inlineStr">
         <is>
@@ -13858,7 +13858,7 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>0.209</v>
+        <v>0.234</v>
       </c>
       <c r="F447" s="2" t="inlineStr">
         <is>
@@ -13888,7 +13888,7 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>0.162</v>
+        <v>0.232</v>
       </c>
       <c r="F448" s="2" t="inlineStr">
         <is>
@@ -13918,7 +13918,7 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>0.206</v>
+        <v>0.2</v>
       </c>
       <c r="F449" s="2" t="inlineStr">
         <is>
@@ -13948,7 +13948,7 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>0.166</v>
+        <v>0.239</v>
       </c>
       <c r="F450" s="2" t="inlineStr">
         <is>
@@ -13978,7 +13978,7 @@
         </is>
       </c>
       <c r="E451" s="2" t="n">
-        <v>0.215</v>
+        <v>0.171</v>
       </c>
       <c r="F451" s="2" t="inlineStr">
         <is>
@@ -14008,7 +14008,7 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>0.169</v>
+        <v>0.242</v>
       </c>
       <c r="F452" s="2" t="inlineStr">
         <is>
@@ -14038,7 +14038,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>0.198</v>
+        <v>0.228</v>
       </c>
       <c r="F453" s="2" t="inlineStr">
         <is>
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>0.177</v>
+        <v>0.201</v>
       </c>
       <c r="F454" s="2" t="inlineStr">
         <is>
@@ -14098,7 +14098,7 @@
         </is>
       </c>
       <c r="E455" s="2" t="n">
-        <v>0.209</v>
+        <v>0.236</v>
       </c>
       <c r="F455" s="2" t="inlineStr">
         <is>
@@ -14128,7 +14128,7 @@
         </is>
       </c>
       <c r="E456" s="2" t="n">
-        <v>0.166</v>
+        <v>0.218</v>
       </c>
       <c r="F456" s="2" t="inlineStr">
         <is>
@@ -14158,7 +14158,7 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>0.2</v>
+        <v>0.199</v>
       </c>
       <c r="F457" s="2" t="inlineStr">
         <is>
@@ -14188,7 +14188,7 @@
         </is>
       </c>
       <c r="E458" s="2" t="n">
-        <v>0.167</v>
+        <v>0.24</v>
       </c>
       <c r="F458" s="2" t="inlineStr">
         <is>
@@ -14218,7 +14218,7 @@
         </is>
       </c>
       <c r="E459" s="2" t="n">
-        <v>0.207</v>
+        <v>0.222</v>
       </c>
       <c r="F459" s="2" t="inlineStr">
         <is>
@@ -14248,7 +14248,7 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>0.194</v>
+        <v>0.204</v>
       </c>
       <c r="F460" s="2" t="inlineStr">
         <is>
@@ -14278,7 +14278,7 @@
         </is>
       </c>
       <c r="E461" s="2" t="n">
-        <v>0.208</v>
+        <v>0.242</v>
       </c>
       <c r="F461" s="2" t="inlineStr">
         <is>
@@ -14308,7 +14308,7 @@
         </is>
       </c>
       <c r="E462" s="2" t="n">
-        <v>0.178</v>
+        <v>0.222</v>
       </c>
       <c r="F462" s="2" t="inlineStr">
         <is>
@@ -14338,7 +14338,7 @@
         </is>
       </c>
       <c r="E463" s="2" t="n">
-        <v>0.198</v>
+        <v>0.2</v>
       </c>
       <c r="F463" s="2" t="inlineStr">
         <is>
@@ -14368,7 +14368,7 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>0.165</v>
+        <v>0.238</v>
       </c>
       <c r="F464" s="2" t="inlineStr">
         <is>
@@ -14428,7 +14428,7 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>0.166</v>
+        <v>0.198</v>
       </c>
       <c r="F466" s="2" t="inlineStr">
         <is>
@@ -14458,7 +14458,7 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="F467" s="2" t="inlineStr">
         <is>
@@ -14488,7 +14488,7 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>0.165</v>
+        <v>0.225</v>
       </c>
       <c r="F468" s="2" t="inlineStr">
         <is>
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>0.2</v>
+        <v>0.197</v>
       </c>
       <c r="F469" s="2" t="inlineStr">
         <is>
@@ -14548,7 +14548,7 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>0.168</v>
+        <v>0.237</v>
       </c>
       <c r="F470" s="2" t="inlineStr">
         <is>
@@ -14578,7 +14578,7 @@
         </is>
       </c>
       <c r="E471" s="2" t="n">
-        <v>0.208</v>
+        <v>0.214</v>
       </c>
       <c r="F471" s="2" t="inlineStr">
         <is>

</xml_diff>